<commit_message>
Update onc tx page
</commit_message>
<xml_diff>
--- a/src/main/webapp/content/files/oncologyTherapies/fda_approved_oncology_therapies.xlsx
+++ b/src/main/webapp/content/files/oncologyTherapies/fda_approved_oncology_therapies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luc2\Desktop\oncokb\oncokb-public\src\main\webapp\content\files\oncologyTherapies\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luc2/Documents/oncokb/oncokb-public/src/main/webapp/content/files/oncologyTherapies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45EF53A-463B-45D4-BCE1-BA0BB0E9A6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3598799-5264-8C48-B722-891F8EC70695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4716" yWindow="576" windowWidth="21480" windowHeight="15456" xr2:uid="{D862B214-800F-AF40-9BAA-60FE1781D5C8}"/>
+    <workbookView xWindow="10600" yWindow="1480" windowWidth="33820" windowHeight="23700" xr2:uid="{D862B214-800F-AF40-9BAA-60FE1781D5C8}"/>
   </bookViews>
   <sheets>
     <sheet name="FDA-Approved Oncology Therapies" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1471" uniqueCount="495">
   <si>
     <t>Year of drug’s first FDA- approval</t>
   </si>
@@ -1722,6 +1722,27 @@
   </si>
   <si>
     <t>Telomerase template antagonist</t>
+  </si>
+  <si>
+    <t>Afamitresgene autoleucel</t>
+  </si>
+  <si>
+    <t>HLA-A*02:01P, -A*02:02P, -A*02:03P, or -A*02:06P positive and MAGE-A4 antigen positive</t>
+  </si>
+  <si>
+    <t>T cell receptor (TCR) therapy</t>
+  </si>
+  <si>
+    <t>MAGE-A4-directed TCR therapy</t>
+  </si>
+  <si>
+    <t>Vorasidenib</t>
+  </si>
+  <si>
+    <t>IDH1 R132H/C/G/S/L, IDH2 R172K/M/W/S/G</t>
+  </si>
+  <si>
+    <t>IDH1/IDH2 inhibitor</t>
   </si>
 </sst>
 </file>
@@ -2148,17 +2169,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B89377A-76F6-CA40-8081-AAD80BFAB6B8}">
-  <dimension ref="A1:H223"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H225"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.5" customWidth="1"/>
-    <col min="2" max="2" width="22.19921875" customWidth="1"/>
-    <col min="3" max="3" width="26.19921875" customWidth="1"/>
-    <col min="4" max="4" width="25.796875" customWidth="1"/>
-    <col min="5" max="5" width="27.296875" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" customWidth="1"/>
+    <col min="3" max="3" width="26.1640625" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2184,7 +2205,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -2207,7 +2228,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -2230,7 +2251,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -2256,7 +2277,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -2279,7 +2300,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
@@ -2302,7 +2323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
         <v>3</v>
       </c>
@@ -2328,7 +2349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
@@ -2351,7 +2372,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A9" s="2" t="s">
         <v>3</v>
       </c>
@@ -2377,7 +2398,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A10" s="2" t="s">
         <v>3</v>
       </c>
@@ -2403,7 +2424,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" s="2" customFormat="1" ht="70" x14ac:dyDescent="0.15">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -2429,7 +2450,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A12" s="2" t="s">
         <v>3</v>
       </c>
@@ -2452,7 +2473,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A13" s="2" t="s">
         <v>3</v>
       </c>
@@ -2475,7 +2496,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A14" s="2" t="s">
         <v>3</v>
       </c>
@@ -2501,7 +2522,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
@@ -2524,7 +2545,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A16" s="2" t="s">
         <v>3</v>
       </c>
@@ -2547,7 +2568,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A17" s="2">
         <v>2002</v>
       </c>
@@ -2573,7 +2594,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A18" s="2">
         <v>2002</v>
       </c>
@@ -2596,7 +2617,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A19" s="2">
         <v>2002</v>
       </c>
@@ -2619,7 +2640,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A20" s="2">
         <v>2003</v>
       </c>
@@ -2643,7 +2664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A21" s="2">
         <v>2003</v>
       </c>
@@ -2666,7 +2687,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A22" s="2">
         <v>2003</v>
       </c>
@@ -2692,7 +2713,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A23" s="2">
         <v>2003</v>
       </c>
@@ -2718,7 +2739,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A24" s="2">
         <v>2004</v>
       </c>
@@ -2741,7 +2762,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A25" s="2">
         <v>2004</v>
       </c>
@@ -2764,7 +2785,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A26" s="2">
         <v>2004</v>
       </c>
@@ -2790,7 +2811,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A27" s="2">
         <v>2004</v>
       </c>
@@ -2813,7 +2834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A28" s="2">
         <v>2004</v>
       </c>
@@ -2839,7 +2860,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A29" s="2">
         <v>2004</v>
       </c>
@@ -2863,7 +2884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A30" s="2">
         <v>2005</v>
       </c>
@@ -2886,7 +2907,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A31" s="2">
         <v>2005</v>
       </c>
@@ -2909,7 +2930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A32" s="2">
         <v>2006</v>
       </c>
@@ -2935,7 +2956,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A33" s="2">
         <v>2006</v>
       </c>
@@ -2958,7 +2979,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A34" s="2">
         <v>2006</v>
       </c>
@@ -2981,7 +3002,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A35" s="2">
         <v>2006</v>
       </c>
@@ -3007,7 +3028,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A36" s="2">
         <v>2006</v>
       </c>
@@ -3033,7 +3054,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A37" s="2">
         <v>2006</v>
       </c>
@@ -3056,7 +3077,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A38" s="2">
         <v>2007</v>
       </c>
@@ -3080,7 +3101,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A39" s="2">
         <v>2007</v>
       </c>
@@ -3106,7 +3127,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A40" s="2">
         <v>2007</v>
       </c>
@@ -3132,7 +3153,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A41" s="2">
         <v>2007</v>
       </c>
@@ -3156,7 +3177,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A42" s="2">
         <v>2008</v>
       </c>
@@ -3179,7 +3200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A43" s="2">
         <v>2008</v>
       </c>
@@ -3202,7 +3223,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A44" s="2">
         <v>2009</v>
       </c>
@@ -3228,7 +3249,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A45" s="2">
         <v>2009</v>
       </c>
@@ -3251,7 +3272,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A46" s="2">
         <v>2009</v>
       </c>
@@ -3274,7 +3295,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A47" s="2">
         <v>2009</v>
       </c>
@@ -3298,7 +3319,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A48" s="2">
         <v>2009</v>
       </c>
@@ -3321,7 +3342,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A49" s="2">
         <v>2010</v>
       </c>
@@ -3344,7 +3365,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A50" s="2">
         <v>2010</v>
       </c>
@@ -3368,7 +3389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A51" s="2">
         <v>2010</v>
       </c>
@@ -3391,7 +3412,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A52" s="2">
         <v>2011</v>
       </c>
@@ -3414,7 +3435,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A53" s="2">
         <v>2011</v>
       </c>
@@ -3438,7 +3459,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A54" s="2">
         <v>2011</v>
       </c>
@@ -3464,7 +3485,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="55" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A55" s="2">
         <v>2011</v>
       </c>
@@ -3490,7 +3511,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A56" s="2">
         <v>2011</v>
       </c>
@@ -3514,7 +3535,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A57" s="2">
         <v>2011</v>
       </c>
@@ -3537,7 +3558,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A58" s="2">
         <v>2011</v>
       </c>
@@ -3560,7 +3581,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A59" s="2">
         <v>2011</v>
       </c>
@@ -3584,7 +3605,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A60" s="2">
         <v>2011</v>
       </c>
@@ -3610,7 +3631,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A61" s="2">
         <v>2012</v>
       </c>
@@ -3633,7 +3654,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A62" s="2">
         <v>2012</v>
       </c>
@@ -3657,7 +3678,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A63" s="2">
         <v>2012</v>
       </c>
@@ -3683,7 +3704,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A64" s="2">
         <v>2012</v>
       </c>
@@ -3706,7 +3727,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A65" s="2">
         <v>2012</v>
       </c>
@@ -3730,7 +3751,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A66" s="2">
         <v>2012</v>
       </c>
@@ -3753,7 +3774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A67" s="2">
         <v>2012</v>
       </c>
@@ -3776,7 +3797,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A68" s="2">
         <v>2012</v>
       </c>
@@ -3802,7 +3823,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A69" s="2">
         <v>2012</v>
       </c>
@@ -3828,7 +3849,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="70" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A70" s="2">
         <v>2012</v>
       </c>
@@ -3854,7 +3875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="71" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A71" s="2">
         <v>2012</v>
       </c>
@@ -3878,7 +3899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A72" s="2">
         <v>2013</v>
       </c>
@@ -3904,7 +3925,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A73" s="2">
         <v>2013</v>
       </c>
@@ -3930,7 +3951,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="74" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A74" s="2">
         <v>2013</v>
       </c>
@@ -3956,7 +3977,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A75" s="2">
         <v>2013</v>
       </c>
@@ -3982,7 +4003,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A76" s="2">
         <v>2013</v>
       </c>
@@ -4005,7 +4026,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A77" s="2">
         <v>2013</v>
       </c>
@@ -4029,7 +4050,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A78" s="2">
         <v>2013</v>
       </c>
@@ -4052,7 +4073,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A79" s="2">
         <v>2013</v>
       </c>
@@ -4078,7 +4099,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A80" s="2">
         <v>2014</v>
       </c>
@@ -4102,7 +4123,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A81" s="2">
         <v>2014</v>
       </c>
@@ -4128,7 +4149,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="82" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A82" s="2">
         <v>2014</v>
       </c>
@@ -4154,7 +4175,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A83" s="2">
         <v>2014</v>
       </c>
@@ -4180,7 +4201,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A84" s="2">
         <v>2014</v>
       </c>
@@ -4203,7 +4224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A85" s="2">
         <v>2014</v>
       </c>
@@ -4226,7 +4247,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A86" s="2">
         <v>2014</v>
       </c>
@@ -4250,7 +4271,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A87" s="2">
         <v>2014</v>
       </c>
@@ -4276,7 +4297,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A88" s="2">
         <v>2014</v>
       </c>
@@ -4302,7 +4323,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:8" s="2" customFormat="1" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" s="2" customFormat="1" ht="56" x14ac:dyDescent="0.15">
       <c r="A89" s="2">
         <v>2014</v>
       </c>
@@ -4328,7 +4349,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A90" s="2">
         <v>2014</v>
       </c>
@@ -4351,7 +4372,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A91" s="2">
         <v>2014</v>
       </c>
@@ -4374,7 +4395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A92" s="2">
         <v>2015</v>
       </c>
@@ -4400,7 +4421,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A93" s="2">
         <v>2015</v>
       </c>
@@ -4426,7 +4447,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A94" s="2">
         <v>2015</v>
       </c>
@@ -4449,7 +4470,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A95" s="2">
         <v>2015</v>
       </c>
@@ -4473,7 +4494,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A96" s="2">
         <v>2015</v>
       </c>
@@ -4496,7 +4517,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A97" s="2">
         <v>2015</v>
       </c>
@@ -4522,7 +4543,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A98" s="2">
         <v>2015</v>
       </c>
@@ -4546,7 +4567,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A99" s="2">
         <v>2015</v>
       </c>
@@ -4569,7 +4590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A100" s="2">
         <v>2015</v>
       </c>
@@ -4592,7 +4613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A101" s="2">
         <v>2015</v>
       </c>
@@ -4618,7 +4639,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="102" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A102" s="2">
         <v>2015</v>
       </c>
@@ -4644,7 +4665,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A103" s="2">
         <v>2015</v>
       </c>
@@ -4667,7 +4688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A104" s="2">
         <v>2015</v>
       </c>
@@ -4691,7 +4712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A105" s="2">
         <v>2015</v>
       </c>
@@ -4714,7 +4735,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A106" s="2">
         <v>2015</v>
       </c>
@@ -4737,7 +4758,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A107" s="2">
         <v>2015</v>
       </c>
@@ -4761,7 +4782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A108" s="2">
         <v>2016</v>
       </c>
@@ -4787,7 +4808,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A109" s="2">
         <v>2016</v>
       </c>
@@ -4810,7 +4831,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A110" s="2">
         <v>2016</v>
       </c>
@@ -4836,7 +4857,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="111" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A111" s="2">
         <v>2016</v>
       </c>
@@ -4859,7 +4880,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A112" s="2">
         <v>2017</v>
       </c>
@@ -4885,7 +4906,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A113" s="2">
         <v>2017</v>
       </c>
@@ -4909,7 +4930,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A114" s="2">
         <v>2017</v>
       </c>
@@ -4932,7 +4953,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A115" s="2">
         <v>2017</v>
       </c>
@@ -4955,7 +4976,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A116" s="2">
         <v>2017</v>
       </c>
@@ -4981,7 +5002,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="117" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A117" s="2">
         <v>2017</v>
       </c>
@@ -5004,7 +5025,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A118" s="2">
         <v>2017</v>
       </c>
@@ -5027,7 +5048,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="119" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A119" s="2">
         <v>2017</v>
       </c>
@@ -5051,7 +5072,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A120" s="2">
         <v>2017</v>
       </c>
@@ -5077,7 +5098,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="121" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A121" s="2">
         <v>2017</v>
       </c>
@@ -5103,7 +5124,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A122" s="2">
         <v>2017</v>
       </c>
@@ -5129,7 +5150,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="123" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A123" s="2">
         <v>2017</v>
       </c>
@@ -5155,7 +5176,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="124" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A124" s="2">
         <v>2017</v>
       </c>
@@ -5181,7 +5202,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="125" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A125" s="2">
         <v>2017</v>
       </c>
@@ -5207,7 +5228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="126" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A126" s="2">
         <v>2017</v>
       </c>
@@ -5230,7 +5251,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="127" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A127" s="2">
         <v>2018</v>
       </c>
@@ -5253,7 +5274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="128" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A128" s="2">
         <v>2018</v>
       </c>
@@ -5279,7 +5300,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="129" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A129" s="2">
         <v>2018</v>
       </c>
@@ -5302,7 +5323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="130" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A130" s="2">
         <v>2018</v>
       </c>
@@ -5328,7 +5349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="131" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A131" s="2">
         <v>2018</v>
       </c>
@@ -5354,7 +5375,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A132" s="2">
         <v>2018</v>
       </c>
@@ -5377,7 +5398,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A133" s="2">
         <v>2018</v>
       </c>
@@ -5403,7 +5424,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="134" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A134" s="2">
         <v>2018</v>
       </c>
@@ -5427,7 +5448,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="135" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A135" s="2">
         <v>2018</v>
       </c>
@@ -5450,7 +5471,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="136" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A136" s="2">
         <v>2018</v>
       </c>
@@ -5476,7 +5497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="137" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A137" s="2">
         <v>2018</v>
       </c>
@@ -5502,7 +5523,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="138" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A138" s="2">
         <v>2018</v>
       </c>
@@ -5528,7 +5549,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="139" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A139" s="2">
         <v>2018</v>
       </c>
@@ -5554,7 +5575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="140" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A140" s="2">
         <v>2018</v>
       </c>
@@ -5578,7 +5599,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="141" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A141" s="2">
         <v>2018</v>
       </c>
@@ -5601,7 +5622,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="142" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A142" s="2">
         <v>2018</v>
       </c>
@@ -5624,7 +5645,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="143" spans="1:8" s="2" customFormat="1" ht="79.2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" s="2" customFormat="1" ht="98" x14ac:dyDescent="0.15">
       <c r="A143" s="2">
         <v>2018</v>
       </c>
@@ -5650,7 +5671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="144" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A144" s="2">
         <v>2019</v>
       </c>
@@ -5676,7 +5697,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="145" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A145" s="2">
         <v>2019</v>
       </c>
@@ -5699,7 +5720,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="146" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A146" s="2">
         <v>2019</v>
       </c>
@@ -5723,7 +5744,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="147" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A147" s="2">
         <v>2019</v>
       </c>
@@ -5749,7 +5770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="148" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A148" s="2">
         <v>2019</v>
       </c>
@@ -5775,7 +5796,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="149" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A149" s="2">
         <v>2019</v>
       </c>
@@ -5799,7 +5820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="150" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A150" s="2">
         <v>2019</v>
       </c>
@@ -5822,7 +5843,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A151" s="2">
         <v>2019</v>
       </c>
@@ -5845,7 +5866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="152" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A152" s="2">
         <v>2019</v>
       </c>
@@ -5869,7 +5890,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A153" s="2">
         <v>2019</v>
       </c>
@@ -5895,7 +5916,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="154" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A154" s="2">
         <v>2019</v>
       </c>
@@ -5918,7 +5939,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A155" s="2">
         <v>2020</v>
       </c>
@@ -5944,7 +5965,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="156" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A156" s="2">
         <v>2020</v>
       </c>
@@ -5970,7 +5991,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A157" s="2">
         <v>2020</v>
       </c>
@@ -5993,7 +6014,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="158" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A158" s="2">
         <v>2020</v>
       </c>
@@ -6017,7 +6038,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="159" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A159" s="2">
         <v>2020</v>
       </c>
@@ -6043,7 +6064,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="160" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A160" s="2">
         <v>2020</v>
       </c>
@@ -6066,7 +6087,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="161" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A161" s="2">
         <v>2020</v>
       </c>
@@ -6092,7 +6113,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A162" s="2">
         <v>2020</v>
       </c>
@@ -6115,7 +6136,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A163" s="2">
         <v>2020</v>
       </c>
@@ -6138,7 +6159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A164" s="2">
         <v>2020</v>
       </c>
@@ -6164,7 +6185,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="165" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A165" s="2">
         <v>2020</v>
       </c>
@@ -6184,7 +6205,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="166" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A166" s="2">
         <v>2020</v>
       </c>
@@ -6210,7 +6231,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="167" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A167" s="2">
         <v>2020</v>
       </c>
@@ -6236,7 +6257,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="168" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A168" s="2">
         <v>2020</v>
       </c>
@@ -6259,7 +6280,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="169" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A169" s="2">
         <v>2020</v>
       </c>
@@ -6285,7 +6306,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="170" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A170" s="2">
         <v>2020</v>
       </c>
@@ -6311,7 +6332,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="171" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A171" s="2">
         <v>2020</v>
       </c>
@@ -6337,7 +6358,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="172" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A172" s="2">
         <v>2020</v>
       </c>
@@ -6363,7 +6384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="173" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A173" s="2">
         <v>2020</v>
       </c>
@@ -6387,7 +6408,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="174" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A174" s="2">
         <v>2020</v>
       </c>
@@ -6413,7 +6434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="175" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A175" s="2">
         <v>2020</v>
       </c>
@@ -6439,7 +6460,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="176" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A176" s="2">
         <v>2021</v>
       </c>
@@ -6465,7 +6486,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A177" s="2">
         <v>2021</v>
       </c>
@@ -6491,7 +6512,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="178" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A178" s="2">
         <v>2021</v>
       </c>
@@ -6517,7 +6538,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="179" spans="1:8" s="2" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A179" s="2">
         <v>2021</v>
       </c>
@@ -6543,7 +6564,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="180" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A180" s="2">
         <v>2021</v>
       </c>
@@ -6566,7 +6587,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A181" s="2">
         <v>2021</v>
       </c>
@@ -6592,7 +6613,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="182" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A182" s="2">
         <v>2021</v>
       </c>
@@ -6616,7 +6637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A183" s="2">
         <v>2021</v>
       </c>
@@ -6639,7 +6660,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="184" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A184" s="2">
         <v>2021</v>
       </c>
@@ -6662,7 +6683,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="185" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A185" s="2">
         <v>2021</v>
       </c>
@@ -6688,7 +6709,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="186" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A186" s="2">
         <v>2021</v>
       </c>
@@ -6711,7 +6732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="187" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A187" s="2">
         <v>2021</v>
       </c>
@@ -6737,7 +6758,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="188" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:8" s="2" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A188" s="2">
         <v>2021</v>
       </c>
@@ -6763,7 +6784,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="189" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A189" s="2">
         <v>2021</v>
       </c>
@@ -6786,7 +6807,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="190" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A190" s="2">
         <v>2021</v>
       </c>
@@ -6809,7 +6830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="191" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A191" s="2">
         <v>2021</v>
       </c>
@@ -6835,7 +6856,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="192" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A192" s="2">
         <v>2021</v>
       </c>
@@ -6858,7 +6879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="193" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A193" s="2">
         <v>2022</v>
       </c>
@@ -6884,7 +6905,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="194" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A194" s="2">
         <v>2022</v>
       </c>
@@ -6908,7 +6929,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="195" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A195" s="2">
         <v>2022</v>
       </c>
@@ -6934,7 +6955,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="196" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A196" s="2">
         <v>2022</v>
       </c>
@@ -6960,7 +6981,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="197" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A197" s="2">
         <v>2022</v>
       </c>
@@ -6984,7 +7005,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="198" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A198" s="2">
         <v>2022</v>
       </c>
@@ -7007,7 +7028,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="199" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A199" s="2">
         <v>2022</v>
       </c>
@@ -7030,7 +7051,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="200" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A200" s="2">
         <v>2022</v>
       </c>
@@ -7056,7 +7077,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="201" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A201" s="2">
         <v>2022</v>
       </c>
@@ -7082,7 +7103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="202" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A202" s="2">
         <v>2022</v>
       </c>
@@ -7108,7 +7129,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="203" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A203" s="2">
         <v>2022</v>
       </c>
@@ -7132,7 +7153,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="204" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A204" s="2">
         <v>2022</v>
       </c>
@@ -7155,7 +7176,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="205" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A205" s="2">
         <v>2023</v>
       </c>
@@ -7181,7 +7202,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="206" spans="1:8" s="2" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:8" s="2" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A206" s="2">
         <v>2023</v>
       </c>
@@ -7207,7 +7228,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="207" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A207" s="2">
         <v>2023</v>
       </c>
@@ -7230,7 +7251,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="208" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A208" s="2">
         <v>2023</v>
       </c>
@@ -7253,7 +7274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="209" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A209" s="2">
         <v>2023</v>
       </c>
@@ -7277,7 +7298,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="210" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A210" s="2">
         <v>2023</v>
       </c>
@@ -7300,7 +7321,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="211" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A211" s="2">
         <v>2023</v>
       </c>
@@ -7323,7 +7344,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="212" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A212" s="2">
         <v>2023</v>
       </c>
@@ -7347,7 +7368,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="213" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A213" s="2">
         <v>2023</v>
       </c>
@@ -7373,7 +7394,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="214" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A214" s="2">
         <v>2023</v>
       </c>
@@ -7399,7 +7420,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="215" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" s="2" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A215" s="2">
         <v>2023</v>
       </c>
@@ -7423,7 +7444,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="216" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A216" s="2">
         <v>2023</v>
       </c>
@@ -7446,7 +7467,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="217" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A217" s="2">
         <v>2023</v>
       </c>
@@ -7469,7 +7490,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="218" spans="1:8" s="2" customFormat="1" ht="13.2" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" s="2" customFormat="1" ht="13" x14ac:dyDescent="0.15">
       <c r="A218" s="2">
         <v>2023</v>
       </c>
@@ -7492,7 +7513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A219" s="2">
         <v>2024</v>
       </c>
@@ -7516,7 +7537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="5">
         <v>2024</v>
       </c>
@@ -7540,7 +7561,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="2">
         <v>2024</v>
       </c>
@@ -7566,7 +7587,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="5">
         <v>2024</v>
       </c>
@@ -7590,7 +7611,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" s="5">
         <v>2024</v>
       </c>
@@ -7612,6 +7633,58 @@
       </c>
       <c r="H223" s="5" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" ht="43" x14ac:dyDescent="0.2">
+      <c r="A224" s="3">
+        <v>2024</v>
+      </c>
+      <c r="B224" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="C224" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="D224" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="E224" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="F224" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G224" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H224" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" ht="29" x14ac:dyDescent="0.2">
+      <c r="A225" s="3">
+        <v>2024</v>
+      </c>
+      <c r="B225" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="D225" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E225" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="F225" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G225" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H225" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -7626,42 +7699,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97AB9D94-D219-C745-BD3C-1D6167799F61}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="153.19921875" customWidth="1"/>
+    <col min="1" max="1" width="153.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="55.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" ht="59" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="42.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="45" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="66" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>468</v>
       </c>

</xml_diff>

<commit_message>
Update precision tx page
</commit_message>
<xml_diff>
--- a/src/main/webapp/content/files/oncologyTherapies/fda_approved_oncology_therapies.xlsx
+++ b/src/main/webapp/content/files/oncologyTherapies/fda_approved_oncology_therapies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cavendk1/Documents/New onc therapies/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luc2/MSK/oncokb/oncokb-pipeline/python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A50A02A-F303-074A-9252-DA2B75C15630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3BF5860-F7FE-8141-A26A-832D3806CA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="880" yWindow="760" windowWidth="29020" windowHeight="17440" xr2:uid="{D862B214-800F-AF40-9BAA-60FE1781D5C8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" xr2:uid="{D862B214-800F-AF40-9BAA-60FE1781D5C8}"/>
   </bookViews>
   <sheets>
     <sheet name="FDA-Approved Oncology Therapies" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1643" uniqueCount="548">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1650" uniqueCount="551">
   <si>
     <t>Year of drug’s first FDA- approval</t>
   </si>
@@ -1895,6 +1895,15 @@
   </si>
   <si>
     <t>Sevabertinib</t>
+  </si>
+  <si>
+    <t>Trastuzumab deruxtecan + Pertuzumab</t>
+  </si>
+  <si>
+    <t>Antibody drug conjugate and monocolonal antibody</t>
+  </si>
+  <si>
+    <t>HER2 (ERBB2)-directed antibody and topoisomerase inhibitor conjugate + anti-HER2 (ERBB2) antibody</t>
   </si>
 </sst>
 </file>
@@ -2015,7 +2024,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2044,13 +2053,10 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2365,7 +2371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B89377A-76F6-CA40-8081-AAD80BFAB6B8}">
-  <dimension ref="A1:I250"/>
+  <dimension ref="A1:I251"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" customWidth="1"/>
@@ -2403,7 +2409,7 @@
       </c>
       <c r="I1" s="11"/>
     </row>
-    <row r="2" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -2505,7 +2511,7 @@
       </c>
       <c r="I5" s="7"/>
     </row>
-    <row r="6" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A6" s="7" t="s">
         <v>3</v>
       </c>
@@ -2530,7 +2536,7 @@
       </c>
       <c r="I6" s="7"/>
     </row>
-    <row r="7" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
@@ -2609,7 +2615,7 @@
       </c>
       <c r="I9" s="7"/>
     </row>
-    <row r="10" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A10" s="7" t="s">
         <v>3</v>
       </c>
@@ -2636,7 +2642,7 @@
       </c>
       <c r="I10" s="7"/>
     </row>
-    <row r="11" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A11" s="7">
         <v>2018</v>
       </c>
@@ -2817,7 +2823,7 @@
       </c>
       <c r="I17" s="7"/>
     </row>
-    <row r="18" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A18" s="7">
         <v>2002</v>
       </c>
@@ -2892,7 +2898,7 @@
       </c>
       <c r="I20" s="7"/>
     </row>
-    <row r="21" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A21" s="7">
         <v>2003</v>
       </c>
@@ -2917,7 +2923,7 @@
       </c>
       <c r="I21" s="7"/>
     </row>
-    <row r="22" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A22" s="7">
         <v>2003</v>
       </c>
@@ -2944,7 +2950,7 @@
       </c>
       <c r="I22" s="7"/>
     </row>
-    <row r="23" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A23" s="7">
         <v>2003</v>
       </c>
@@ -2971,7 +2977,7 @@
       </c>
       <c r="I23" s="7"/>
     </row>
-    <row r="24" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A24" s="7">
         <v>2004</v>
       </c>
@@ -3048,7 +3054,7 @@
       </c>
       <c r="I26" s="7"/>
     </row>
-    <row r="27" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A27" s="7">
         <v>2004</v>
       </c>
@@ -3073,7 +3079,7 @@
       </c>
       <c r="I27" s="7"/>
     </row>
-    <row r="28" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A28" s="7">
         <v>2004</v>
       </c>
@@ -3125,7 +3131,7 @@
       </c>
       <c r="I29" s="7"/>
     </row>
-    <row r="30" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A30" s="7">
         <v>2005</v>
       </c>
@@ -3177,7 +3183,7 @@
       </c>
       <c r="I31" s="7"/>
     </row>
-    <row r="32" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A32" s="7">
         <v>2019</v>
       </c>
@@ -3202,7 +3208,7 @@
       </c>
       <c r="I32" s="7"/>
     </row>
-    <row r="33" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A33" s="7">
         <v>2006</v>
       </c>
@@ -3512,7 +3518,7 @@
       </c>
       <c r="I44" s="7"/>
     </row>
-    <row r="45" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A45" s="7">
         <v>2009</v>
       </c>
@@ -3537,7 +3543,7 @@
       </c>
       <c r="I45" s="7"/>
     </row>
-    <row r="46" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A46" s="7">
         <v>2019</v>
       </c>
@@ -3737,7 +3743,7 @@
       </c>
       <c r="I53" s="7"/>
     </row>
-    <row r="54" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A54" s="7">
         <v>2011</v>
       </c>
@@ -3764,7 +3770,7 @@
       </c>
       <c r="I54" s="7"/>
     </row>
-    <row r="55" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A55" s="7">
         <v>2020</v>
       </c>
@@ -3791,7 +3797,7 @@
       </c>
       <c r="I55" s="7"/>
     </row>
-    <row r="56" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A56" s="7">
         <v>2011</v>
       </c>
@@ -3816,7 +3822,7 @@
       </c>
       <c r="I56" s="7"/>
     </row>
-    <row r="57" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A57" s="7">
         <v>2011</v>
       </c>
@@ -3841,7 +3847,7 @@
       </c>
       <c r="I57" s="7"/>
     </row>
-    <row r="58" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A58" s="7">
         <v>2011</v>
       </c>
@@ -3893,7 +3899,7 @@
       </c>
       <c r="I59" s="7"/>
     </row>
-    <row r="60" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A60" s="7">
         <v>2011</v>
       </c>
@@ -3970,7 +3976,7 @@
       </c>
       <c r="I62" s="7"/>
     </row>
-    <row r="63" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A63" s="7">
         <v>2021</v>
       </c>
@@ -4022,7 +4028,7 @@
       </c>
       <c r="I64" s="7"/>
     </row>
-    <row r="65" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A65" s="7">
         <v>2012</v>
       </c>
@@ -4072,7 +4078,7 @@
       </c>
       <c r="I66" s="7"/>
     </row>
-    <row r="67" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A67" s="7">
         <v>2012</v>
       </c>
@@ -4097,7 +4103,7 @@
       </c>
       <c r="I67" s="7"/>
     </row>
-    <row r="68" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A68" s="7">
         <v>2012</v>
       </c>
@@ -4124,7 +4130,7 @@
       </c>
       <c r="I68" s="7"/>
     </row>
-    <row r="69" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A69" s="7">
         <v>2006</v>
       </c>
@@ -4201,7 +4207,7 @@
       </c>
       <c r="I71" s="7"/>
     </row>
-    <row r="72" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A72" s="7">
         <v>2013</v>
       </c>
@@ -4255,7 +4261,7 @@
       </c>
       <c r="I73" s="7"/>
     </row>
-    <row r="74" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A74" s="7">
         <v>2013</v>
       </c>
@@ -4282,7 +4288,7 @@
       </c>
       <c r="I74" s="7"/>
     </row>
-    <row r="75" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A75" s="7">
         <v>2013</v>
       </c>
@@ -4309,7 +4315,7 @@
       </c>
       <c r="I75" s="7"/>
     </row>
-    <row r="76" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A76" s="7">
         <v>2013</v>
       </c>
@@ -4384,7 +4390,7 @@
       </c>
       <c r="I78" s="7"/>
     </row>
-    <row r="79" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A79" s="7">
         <v>2013</v>
       </c>
@@ -4463,7 +4469,7 @@
       </c>
       <c r="I81" s="7"/>
     </row>
-    <row r="82" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A82" s="7">
         <v>2014</v>
       </c>
@@ -4592,7 +4598,7 @@
       </c>
       <c r="I86" s="7"/>
     </row>
-    <row r="87" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A87" s="7">
         <v>2014</v>
       </c>
@@ -4698,7 +4704,7 @@
       </c>
       <c r="I90" s="7"/>
     </row>
-    <row r="91" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A91" s="7">
         <v>2014</v>
       </c>
@@ -4723,7 +4729,7 @@
       </c>
       <c r="I91" s="7"/>
     </row>
-    <row r="92" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A92" s="7">
         <v>2015</v>
       </c>
@@ -4777,7 +4783,7 @@
       </c>
       <c r="I93" s="7"/>
     </row>
-    <row r="94" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A94" s="7">
         <v>2015</v>
       </c>
@@ -4827,7 +4833,7 @@
       </c>
       <c r="I95" s="7"/>
     </row>
-    <row r="96" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A96" s="7">
         <v>2015</v>
       </c>
@@ -4879,7 +4885,7 @@
       </c>
       <c r="I97" s="7"/>
     </row>
-    <row r="98" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A98" s="7">
         <v>2015</v>
       </c>
@@ -4904,7 +4910,7 @@
       </c>
       <c r="I98" s="7"/>
     </row>
-    <row r="99" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A99" s="7">
         <v>2021</v>
       </c>
@@ -4981,7 +4987,7 @@
       </c>
       <c r="I101" s="7"/>
     </row>
-    <row r="102" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A102" s="7">
         <v>2015</v>
       </c>
@@ -5108,7 +5114,7 @@
       </c>
       <c r="I106" s="7"/>
     </row>
-    <row r="107" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A107" s="7">
         <v>2015</v>
       </c>
@@ -5133,7 +5139,7 @@
       </c>
       <c r="I107" s="7"/>
     </row>
-    <row r="108" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A108" s="7">
         <v>2016</v>
       </c>
@@ -5237,7 +5243,7 @@
       </c>
       <c r="I111" s="7"/>
     </row>
-    <row r="112" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A112" s="7">
         <v>2017</v>
       </c>
@@ -5264,7 +5270,7 @@
       </c>
       <c r="I112" s="7"/>
     </row>
-    <row r="113" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A113" s="7">
         <v>2017</v>
       </c>
@@ -5289,7 +5295,7 @@
       </c>
       <c r="I113" s="7"/>
     </row>
-    <row r="114" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A114" s="7">
         <v>2017</v>
       </c>
@@ -5339,7 +5345,7 @@
       </c>
       <c r="I115" s="7"/>
     </row>
-    <row r="116" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A116" s="7">
         <v>2017</v>
       </c>
@@ -5391,7 +5397,7 @@
       </c>
       <c r="I117" s="7"/>
     </row>
-    <row r="118" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A118" s="7">
         <v>2017</v>
       </c>
@@ -5416,7 +5422,7 @@
       </c>
       <c r="I118" s="7"/>
     </row>
-    <row r="119" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A119" s="7">
         <v>2017</v>
       </c>
@@ -5470,7 +5476,7 @@
       </c>
       <c r="I120" s="7"/>
     </row>
-    <row r="121" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A121" s="7">
         <v>2017</v>
       </c>
@@ -5524,7 +5530,7 @@
       </c>
       <c r="I122" s="7"/>
     </row>
-    <row r="123" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A123" s="7">
         <v>2017</v>
       </c>
@@ -5578,7 +5584,7 @@
       </c>
       <c r="I124" s="7"/>
     </row>
-    <row r="125" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A125" s="7">
         <v>2017</v>
       </c>
@@ -5707,7 +5713,7 @@
       </c>
       <c r="I129" s="7"/>
     </row>
-    <row r="130" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A130" s="7">
         <v>2018</v>
       </c>
@@ -5734,7 +5740,7 @@
       </c>
       <c r="I130" s="7"/>
     </row>
-    <row r="131" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A131" s="7">
         <v>2018</v>
       </c>
@@ -5786,7 +5792,7 @@
       </c>
       <c r="I132" s="7"/>
     </row>
-    <row r="133" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A133" s="7">
         <v>2011</v>
       </c>
@@ -5888,7 +5894,7 @@
       </c>
       <c r="I136" s="7"/>
     </row>
-    <row r="137" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A137" s="7">
         <v>2018</v>
       </c>
@@ -5915,7 +5921,7 @@
       </c>
       <c r="I137" s="7"/>
     </row>
-    <row r="138" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A138" s="7">
         <v>2012</v>
       </c>
@@ -5967,7 +5973,7 @@
       </c>
       <c r="I139" s="7"/>
     </row>
-    <row r="140" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A140" s="7">
         <v>2018</v>
       </c>
@@ -5992,7 +5998,7 @@
       </c>
       <c r="I140" s="7"/>
     </row>
-    <row r="141" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A141" s="7">
         <v>2018</v>
       </c>
@@ -6017,7 +6023,7 @@
       </c>
       <c r="I141" s="7"/>
     </row>
-    <row r="142" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A142" s="7">
         <v>2018</v>
       </c>
@@ -6121,7 +6127,7 @@
       </c>
       <c r="I145" s="7"/>
     </row>
-    <row r="146" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A146" s="7">
         <v>2019</v>
       </c>
@@ -6146,7 +6152,7 @@
       </c>
       <c r="I146" s="7"/>
     </row>
-    <row r="147" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A147" s="7">
         <v>2015</v>
       </c>
@@ -6171,7 +6177,7 @@
       </c>
       <c r="I147" s="7"/>
     </row>
-    <row r="148" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A148" s="7">
         <v>2006</v>
       </c>
@@ -6198,7 +6204,7 @@
       </c>
       <c r="I148" s="7"/>
     </row>
-    <row r="149" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A149" s="7">
         <v>2012</v>
       </c>
@@ -6252,7 +6258,7 @@
       </c>
       <c r="I150" s="7"/>
     </row>
-    <row r="151" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A151" s="7">
         <v>2019</v>
       </c>
@@ -6329,7 +6335,7 @@
       </c>
       <c r="I153" s="7"/>
     </row>
-    <row r="154" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="154" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A154" s="7">
         <v>2019</v>
       </c>
@@ -6381,7 +6387,7 @@
       </c>
       <c r="I155" s="7"/>
     </row>
-    <row r="156" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="156" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A156" s="7">
         <v>2012</v>
       </c>
@@ -6408,7 +6414,7 @@
       </c>
       <c r="I156" s="7"/>
     </row>
-    <row r="157" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="157" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A157" s="7">
         <v>2020</v>
       </c>
@@ -6458,7 +6464,7 @@
       </c>
       <c r="I158" s="7"/>
     </row>
-    <row r="159" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="159" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A159" s="7">
         <v>2020</v>
       </c>
@@ -6510,7 +6516,7 @@
       </c>
       <c r="I160" s="7"/>
     </row>
-    <row r="161" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="161" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A161" s="7">
         <v>2020</v>
       </c>
@@ -6537,7 +6543,7 @@
       </c>
       <c r="I161" s="7"/>
     </row>
-    <row r="162" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="162" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A162" s="7">
         <v>2020</v>
       </c>
@@ -6666,7 +6672,7 @@
       </c>
       <c r="I166" s="7"/>
     </row>
-    <row r="167" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="167" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A167" s="7">
         <v>2020</v>
       </c>
@@ -6718,7 +6724,7 @@
       </c>
       <c r="I168" s="7"/>
     </row>
-    <row r="169" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="169" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A169" s="7">
         <v>2020</v>
       </c>
@@ -6745,7 +6751,7 @@
       </c>
       <c r="I169" s="7"/>
     </row>
-    <row r="170" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="170" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A170" s="7">
         <v>2020</v>
       </c>
@@ -6799,7 +6805,7 @@
       </c>
       <c r="I171" s="7"/>
     </row>
-    <row r="172" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="172" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A172" s="7">
         <v>2020</v>
       </c>
@@ -6826,7 +6832,7 @@
       </c>
       <c r="I172" s="7"/>
     </row>
-    <row r="173" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="173" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A173" s="7">
         <v>2020</v>
       </c>
@@ -7038,7 +7044,7 @@
       </c>
       <c r="I180" s="7"/>
     </row>
-    <row r="181" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="181" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A181" s="7">
         <v>2021</v>
       </c>
@@ -7082,7 +7088,7 @@
       <c r="F182" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G182" s="15" t="s">
+      <c r="G182" s="2" t="s">
         <v>7</v>
       </c>
       <c r="H182" s="7" t="s">
@@ -7090,7 +7096,7 @@
       </c>
       <c r="I182" s="7"/>
     </row>
-    <row r="183" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="183" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A183" s="7">
         <v>2021</v>
       </c>
@@ -7140,7 +7146,7 @@
       </c>
       <c r="I184" s="7"/>
     </row>
-    <row r="185" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="185" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A185" s="7">
         <v>2021</v>
       </c>
@@ -7219,7 +7225,7 @@
       </c>
       <c r="I187" s="7"/>
     </row>
-    <row r="188" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="188" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A188" s="7">
         <v>2021</v>
       </c>
@@ -7246,7 +7252,7 @@
       </c>
       <c r="I188" s="7"/>
     </row>
-    <row r="189" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="189" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A189" s="7">
         <v>2021</v>
       </c>
@@ -7298,7 +7304,7 @@
       </c>
       <c r="I190" s="7"/>
     </row>
-    <row r="191" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="191" spans="1:9" s="5" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A191" s="7">
         <v>2021</v>
       </c>
@@ -7404,7 +7410,7 @@
       </c>
       <c r="I194" s="7"/>
     </row>
-    <row r="195" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="195" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A195" s="7">
         <v>2022</v>
       </c>
@@ -7431,7 +7437,7 @@
       </c>
       <c r="I195" s="7"/>
     </row>
-    <row r="196" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="196" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A196" s="7">
         <v>2022</v>
       </c>
@@ -7587,7 +7593,7 @@
       </c>
       <c r="I201" s="7"/>
     </row>
-    <row r="202" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="202" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A202" s="7">
         <v>2022</v>
       </c>
@@ -7793,7 +7799,7 @@
       </c>
       <c r="I209" s="7"/>
     </row>
-    <row r="210" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="210" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A210" s="7">
         <v>2023</v>
       </c>
@@ -7843,7 +7849,7 @@
       </c>
       <c r="I211" s="7"/>
     </row>
-    <row r="212" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="212" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A212" s="7">
         <v>2023</v>
       </c>
@@ -7920,7 +7926,7 @@
       </c>
       <c r="I214" s="7"/>
     </row>
-    <row r="215" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="215" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A215" s="7">
         <v>2023</v>
       </c>
@@ -7970,7 +7976,7 @@
       </c>
       <c r="I216" s="7"/>
     </row>
-    <row r="217" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
+    <row r="217" spans="1:9" s="5" customFormat="1" ht="28" x14ac:dyDescent="0.15">
       <c r="A217" s="7">
         <v>2023</v>
       </c>
@@ -8027,6 +8033,7 @@
       <c r="B219" s="2" t="s">
         <v>458</v>
       </c>
+      <c r="C219" s="15"/>
       <c r="D219" s="2" t="s">
         <v>35</v>
       </c>
@@ -8193,7 +8200,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="226" spans="1:9" s="4" customFormat="1" ht="28" x14ac:dyDescent="0.15">
+    <row r="226" spans="1:9" s="4" customFormat="1" ht="42" x14ac:dyDescent="0.15">
       <c r="A226" s="7">
         <v>2024</v>
       </c>
@@ -8220,7 +8227,7 @@
       </c>
       <c r="I226" s="7"/>
     </row>
-    <row r="227" spans="1:9" ht="29" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:9" ht="43" x14ac:dyDescent="0.2">
       <c r="A227" s="7">
         <v>2024</v>
       </c>
@@ -8246,7 +8253,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="29" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:9" ht="43" x14ac:dyDescent="0.2">
       <c r="A228" s="7">
         <v>2024</v>
       </c>
@@ -8329,7 +8336,7 @@
       <c r="B231" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="C231" s="14" t="s">
+      <c r="C231" s="2" t="s">
         <v>545</v>
       </c>
       <c r="D231" s="2" t="s">
@@ -8384,10 +8391,10 @@
       <c r="C233" s="2" t="s">
         <v>499</v>
       </c>
-      <c r="D233" s="14" t="s">
+      <c r="D233" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="E233" s="14" t="s">
+      <c r="E233" s="2" t="s">
         <v>532</v>
       </c>
       <c r="F233" s="7" t="s">
@@ -8400,13 +8407,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:9" ht="29" x14ac:dyDescent="0.2">
       <c r="A234" s="7">
         <v>2024</v>
       </c>
       <c r="B234" s="2" t="s">
         <v>507</v>
       </c>
+      <c r="C234" s="15"/>
       <c r="D234" s="2" t="s">
         <v>109</v>
       </c>
@@ -8423,7 +8431,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:9" ht="29" x14ac:dyDescent="0.2">
       <c r="A235" s="7">
         <v>2024</v>
       </c>
@@ -8449,7 +8457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="29" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:9" ht="43" x14ac:dyDescent="0.2">
       <c r="A236" s="7">
         <v>2025</v>
       </c>
@@ -8476,283 +8484,283 @@
       </c>
     </row>
     <row r="237" spans="1:9" ht="29" x14ac:dyDescent="0.2">
-      <c r="A237" s="5">
+      <c r="A237" s="7">
         <v>2025</v>
       </c>
-      <c r="B237" s="14" t="s">
+      <c r="B237" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="C237" s="14" t="s">
+      <c r="C237" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="D237" s="14" t="s">
+      <c r="D237" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E237" s="14" t="s">
+      <c r="E237" s="2" t="s">
         <v>517</v>
       </c>
-      <c r="F237" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G237" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H237" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A238" s="5">
+      <c r="F237" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G237" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H237" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="238" spans="1:9" ht="29" x14ac:dyDescent="0.2">
+      <c r="A238" s="7">
         <v>2025</v>
       </c>
-      <c r="B238" s="14" t="s">
+      <c r="B238" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="C238" s="14" t="s">
+      <c r="C238" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="D238" s="14" t="s">
+      <c r="D238" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E238" s="14" t="s">
+      <c r="E238" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="F238" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G238" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H238" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A239" s="5">
+      <c r="F238" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G238" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H238" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="239" spans="1:9" ht="29" x14ac:dyDescent="0.2">
+      <c r="A239" s="7">
         <v>2025</v>
       </c>
-      <c r="B239" s="14" t="s">
+      <c r="B239" s="2" t="s">
         <v>515</v>
       </c>
-      <c r="C239" s="12"/>
-      <c r="D239" s="14" t="s">
+      <c r="C239" s="15"/>
+      <c r="D239" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E239" s="14" t="s">
+      <c r="E239" s="2" t="s">
         <v>516</v>
       </c>
-      <c r="F239" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G239" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H239" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="240" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A240" s="5">
+      <c r="F239" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G239" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H239" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="240" spans="1:9" s="9" customFormat="1" ht="29" x14ac:dyDescent="0.2">
+      <c r="A240" s="7">
         <v>2025</v>
       </c>
-      <c r="B240" s="14" t="s">
+      <c r="B240" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="C240" s="12"/>
-      <c r="D240" s="14" t="s">
+      <c r="C240" s="15"/>
+      <c r="D240" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E240" s="14" t="s">
+      <c r="E240" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="F240" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G240" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H240" s="5" t="s">
+      <c r="F240" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G240" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H240" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="241" spans="1:9" s="9" customFormat="1" ht="29" x14ac:dyDescent="0.2">
-      <c r="A241" s="5">
+      <c r="A241" s="7">
         <v>2025</v>
       </c>
-      <c r="B241" s="14" t="s">
+      <c r="B241" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="C241" s="14" t="s">
+      <c r="C241" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="D241" s="14" t="s">
+      <c r="D241" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E241" s="14" t="s">
+      <c r="E241" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="F241" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G241" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H241" s="5" t="s">
+      <c r="F241" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G241" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H241" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="242" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A242" s="5">
+      <c r="A242" s="7">
         <v>2025</v>
       </c>
-      <c r="B242" s="14" t="s">
+      <c r="B242" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="C242" s="14" t="s">
+      <c r="C242" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="D242" s="14" t="s">
+      <c r="D242" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E242" s="14" t="s">
+      <c r="E242" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="F242" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G242" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H242" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="243" spans="1:9" s="9" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A243" s="5">
+      <c r="F242" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G242" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H242" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="243" spans="1:9" s="9" customFormat="1" ht="29" x14ac:dyDescent="0.2">
+      <c r="A243" s="7">
         <v>2025</v>
       </c>
-      <c r="B243" s="14" t="s">
+      <c r="B243" s="2" t="s">
         <v>523</v>
       </c>
-      <c r="C243" s="14" t="s">
+      <c r="C243" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="D243" s="14" t="s">
+      <c r="D243" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E243" s="14" t="s">
+      <c r="E243" s="2" t="s">
         <v>524</v>
       </c>
-      <c r="F243" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G243" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H243" s="5" t="s">
+      <c r="F243" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G243" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H243" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="244" spans="1:9" s="5" customFormat="1" ht="14" x14ac:dyDescent="0.15">
-      <c r="A244" s="5">
+      <c r="A244" s="7">
         <v>2025</v>
       </c>
-      <c r="B244" s="14" t="s">
+      <c r="B244" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="C244" s="14"/>
-      <c r="D244" s="14" t="s">
+      <c r="C244" s="2"/>
+      <c r="D244" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="E244" s="14" t="s">
+      <c r="E244" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="F244" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G244" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H244" s="5" t="s">
+      <c r="F244" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G244" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H244" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="245" spans="1:9" s="5" customFormat="1" ht="13" x14ac:dyDescent="0.15">
-      <c r="A245" s="5">
+      <c r="A245" s="7">
         <v>2025</v>
       </c>
-      <c r="B245" s="5" t="s">
+      <c r="B245" s="7" t="s">
         <v>533</v>
       </c>
-      <c r="C245" s="5" t="s">
+      <c r="C245" s="7" t="s">
         <v>389</v>
       </c>
-      <c r="D245" s="5" t="s">
+      <c r="D245" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E245" s="5" t="s">
+      <c r="E245" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F245" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G245" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H245" s="5" t="s">
+      <c r="F245" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G245" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H245" s="7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="246" spans="1:9" ht="43" x14ac:dyDescent="0.2">
-      <c r="A246" s="5">
+      <c r="A246" s="7">
         <v>2025</v>
       </c>
-      <c r="B246" s="5" t="s">
+      <c r="B246" s="7" t="s">
         <v>534</v>
       </c>
-      <c r="C246" s="14" t="s">
+      <c r="C246" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="D246" s="5" t="s">
+      <c r="D246" s="7" t="s">
         <v>535</v>
       </c>
-      <c r="E246" s="5" t="s">
+      <c r="E246" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="F246" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G246" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H246" s="5" t="s">
+      <c r="F246" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G246" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H246" s="7" t="s">
         <v>6</v>
       </c>
       <c r="I246" s="6"/>
     </row>
-    <row r="247" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A247" s="5">
+    <row r="247" spans="1:9" s="14" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A247" s="7">
         <v>2025</v>
       </c>
-      <c r="B247" s="5" t="s">
+      <c r="B247" s="7" t="s">
         <v>538</v>
       </c>
-      <c r="C247" s="5" t="s">
+      <c r="C247" s="7" t="s">
         <v>539</v>
       </c>
-      <c r="D247" s="5" t="s">
+      <c r="D247" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="E247" s="5" t="s">
+      <c r="E247" s="7" t="s">
         <v>540</v>
       </c>
-      <c r="F247" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="G247" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H247" s="5" t="s">
+      <c r="F247" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G247" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H247" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -8831,6 +8839,32 @@
         <v>6</v>
       </c>
       <c r="H250" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="251" spans="1:9" s="4" customFormat="1" ht="42" x14ac:dyDescent="0.15">
+      <c r="A251" s="7">
+        <v>2025</v>
+      </c>
+      <c r="B251" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="C251" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="D251" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="E251" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="F251" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G251" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H251" s="7" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>